<commit_message>
validation and updating all relevant figures
</commit_message>
<xml_diff>
--- a/02_Data_Analysis/data/validation_candidates.xlsx
+++ b/02_Data_Analysis/data/validation_candidates.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -38,7 +38,13 @@
     <t xml:space="preserve">Bi_features_score</t>
   </si>
   <si>
-    <t xml:space="preserve">multibiophys_distance</t>
+    <t xml:space="preserve">Bi_feature_rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multibiophys_similarity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multibiophys_category</t>
   </si>
   <si>
     <t xml:space="preserve">P43357_KVAELVHFL</t>
@@ -50,6 +56,9 @@
     <t xml:space="preserve">Intact</t>
   </si>
   <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
     <t xml:space="preserve">P43362_KVAELVHFL</t>
   </si>
   <si>
@@ -62,6 +71,9 @@
     <t xml:space="preserve">P43360_KVAKLVHFL</t>
   </si>
   <si>
+    <t xml:space="preserve">Moderate</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q9NUL7_KVAELVHIL</t>
   </si>
   <si>
@@ -120,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve">High_Disagreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
   </si>
   <si>
     <t xml:space="preserve">Q15546_KVVELFFYL</t>
@@ -521,16 +536,22 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -547,19 +568,25 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>0</v>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -576,19 +603,25 @@
       <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
-        <v>0</v>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -605,19 +638,25 @@
       <c r="H4" t="n">
         <v>0.957142857142857</v>
       </c>
-      <c r="I4" t="n">
-        <v>0.305435130800666</v>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.876681504988593</v>
+      </c>
+      <c r="K4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -634,19 +673,25 @@
       <c r="H5" t="n">
         <v>0.942857142857143</v>
       </c>
-      <c r="I5" t="n">
-        <v>1.03878013211271</v>
+      <c r="I5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.580595715351778</v>
+      </c>
+      <c r="K5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -663,19 +708,25 @@
       <c r="H6" t="n">
         <v>0.914285714285714</v>
       </c>
-      <c r="I6" t="n">
-        <v>0.842531899794821</v>
+      <c r="I6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.659830335791969</v>
+      </c>
+      <c r="K6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D7" t="n">
         <v>6</v>
@@ -692,19 +743,25 @@
       <c r="H7" t="n">
         <v>0.9</v>
       </c>
-      <c r="I7" t="n">
-        <v>0.152395601799665</v>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.938470744308201</v>
+      </c>
+      <c r="K7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
@@ -721,19 +778,25 @@
       <c r="H8" t="n">
         <v>0.885714285714286</v>
       </c>
-      <c r="I8" t="n">
-        <v>0.153396495929034</v>
+      <c r="I8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.938066636380681</v>
+      </c>
+      <c r="K8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D9" t="n">
         <v>7</v>
@@ -750,19 +813,25 @@
       <c r="H9" t="n">
         <v>0.885714285714286</v>
       </c>
-      <c r="I9" t="n">
-        <v>0.656475048957595</v>
+      <c r="I9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.734950217292379</v>
+      </c>
+      <c r="K9" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D10" t="n">
         <v>7</v>
@@ -779,19 +848,25 @@
       <c r="H10" t="n">
         <v>0.885714285714286</v>
       </c>
-      <c r="I10" t="n">
-        <v>0.647000770298773</v>
+      <c r="I10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.738775428172549</v>
+      </c>
+      <c r="K10" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11" t="n">
         <v>10</v>
@@ -808,19 +883,25 @@
       <c r="H11" t="n">
         <v>0.871428571428571</v>
       </c>
-      <c r="I11" t="n">
-        <v>0.660330175081297</v>
+      <c r="I11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.733393721972382</v>
+      </c>
+      <c r="K11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D12" t="n">
         <v>10</v>
@@ -837,19 +918,25 @@
       <c r="H12" t="n">
         <v>0.871428571428571</v>
       </c>
-      <c r="I12" t="n">
-        <v>0.508276535761413</v>
+      <c r="I12" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.794784911364321</v>
+      </c>
+      <c r="K12" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D13" t="n">
         <v>12</v>
@@ -866,19 +953,25 @@
       <c r="H13" t="n">
         <v>0.857142857142857</v>
       </c>
-      <c r="I13" t="n">
-        <v>0.775710737568042</v>
+      <c r="I13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.686809174601762</v>
+      </c>
+      <c r="K13" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14" t="n">
         <v>13</v>
@@ -895,19 +988,25 @@
       <c r="H14" t="n">
         <v>0.842857142857143</v>
       </c>
-      <c r="I14" t="n">
-        <v>0.254153070314338</v>
+      <c r="I14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.897386479245091</v>
+      </c>
+      <c r="K14" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D15" t="n">
         <v>14</v>
@@ -924,19 +1023,25 @@
       <c r="H15" t="n">
         <v>0.828571428571429</v>
       </c>
-      <c r="I15" t="n">
-        <v>1.11960337559575</v>
+      <c r="I15" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.547963579283666</v>
+      </c>
+      <c r="K15" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D16" t="n">
         <v>14</v>
@@ -953,19 +1058,25 @@
       <c r="H16" t="n">
         <v>0.828571428571429</v>
       </c>
-      <c r="I16" t="n">
-        <v>0.841266308799413</v>
+      <c r="I16" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.66034131426535</v>
+      </c>
+      <c r="K16" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D17" t="n">
         <v>14</v>
@@ -982,19 +1093,25 @@
       <c r="H17" t="n">
         <v>0.828571428571429</v>
       </c>
-      <c r="I17" t="n">
-        <v>0.212614283122135</v>
+      <c r="I17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.914157636864431</v>
+      </c>
+      <c r="K17" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D18" t="n">
         <v>18</v>
@@ -1011,19 +1128,25 @@
       <c r="H18" t="n">
         <v>0.814285714285714</v>
       </c>
-      <c r="I18" t="n">
-        <v>0.241683173452397</v>
+      <c r="I18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.902421161764849</v>
+      </c>
+      <c r="K18" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D19" t="n">
         <v>30</v>
@@ -1040,19 +1163,25 @@
       <c r="H19" t="n">
         <v>0.757142857142857</v>
       </c>
-      <c r="I19" t="n">
-        <v>0.152318588917098</v>
+      <c r="I19" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.938501838022764</v>
+      </c>
+      <c r="K19" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D20" t="n">
         <v>43</v>
@@ -1069,19 +1198,25 @@
       <c r="H20" t="n">
         <v>0.728571428571429</v>
       </c>
-      <c r="I20" t="n">
-        <v>0.155529900117394</v>
+      <c r="I20" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.937205280998705</v>
+      </c>
+      <c r="K20" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" t="s">
         <v>33</v>
       </c>
-      <c r="B21" t="s">
-        <v>29</v>
-      </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D21" t="n">
         <v>43</v>
@@ -1098,19 +1233,25 @@
       <c r="H21" t="n">
         <v>0.728571428571429</v>
       </c>
-      <c r="I21" t="n">
-        <v>0.177954951081834</v>
+      <c r="I21" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.928151235616828</v>
+      </c>
+      <c r="K21" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D22" t="n">
         <v>43</v>
@@ -1127,19 +1268,25 @@
       <c r="H22" t="n">
         <v>0.728571428571429</v>
       </c>
-      <c r="I22" t="n">
-        <v>1.6680569749616</v>
+      <c r="I22" t="s">
+        <v>14</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.326527124740635</v>
+      </c>
+      <c r="K22" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D23" t="n">
         <v>74</v>
@@ -1156,19 +1303,25 @@
       <c r="H23" t="n">
         <v>0.7</v>
       </c>
-      <c r="I23" t="n">
-        <v>1.56317177653801</v>
+      <c r="I23" t="s">
+        <v>14</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.368874201138379</v>
+      </c>
+      <c r="K23" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D24" t="n">
         <v>92</v>
@@ -1185,19 +1338,25 @@
       <c r="H24" t="n">
         <v>0.685714285714286</v>
       </c>
-      <c r="I24" t="n">
-        <v>2.10313682204245</v>
+      <c r="I24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.150864974119138</v>
+      </c>
+      <c r="K24" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B25" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D25" t="n">
         <v>108</v>
@@ -1214,19 +1373,25 @@
       <c r="H25" t="n">
         <v>0.671428571428571</v>
       </c>
-      <c r="I25" t="n">
-        <v>1.62437270043123</v>
+      <c r="I25" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.344164516276539</v>
+      </c>
+      <c r="K25" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D26" t="n">
         <v>238</v>
@@ -1243,19 +1408,25 @@
       <c r="H26" t="n">
         <v>0.6</v>
       </c>
-      <c r="I26" t="n">
-        <v>0.199674423969787</v>
+      <c r="I26" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.919382065214058</v>
+      </c>
+      <c r="K26" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D27" t="n">
         <v>832</v>
@@ -1272,19 +1443,25 @@
       <c r="H27" t="n">
         <v>0.307857142857143</v>
       </c>
-      <c r="I27" t="n">
-        <v>0.173065554247307</v>
+      <c r="I27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.930125314556493</v>
+      </c>
+      <c r="K27" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D28" t="n">
         <v>857</v>
@@ -1301,19 +1478,25 @@
       <c r="H28" t="n">
         <v>0.293571428571429</v>
       </c>
-      <c r="I28" t="n">
-        <v>0.240420169825188</v>
+      <c r="I28" t="s">
+        <v>40</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.902931095596275</v>
+      </c>
+      <c r="K28" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D29" t="n">
         <v>1094</v>
@@ -1330,19 +1513,25 @@
       <c r="H29" t="n">
         <v>0.2</v>
       </c>
-      <c r="I29" t="n">
-        <v>0.251291504147878</v>
+      <c r="I29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.898541827787017</v>
+      </c>
+      <c r="K29" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C30" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D30" t="n">
         <v>1209</v>
@@ -1359,19 +1548,25 @@
       <c r="H30" t="n">
         <v>0.128571428571429</v>
       </c>
-      <c r="I30" t="n">
-        <v>0.181132690141069</v>
+      <c r="I30" t="s">
+        <v>40</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.926868233241507</v>
+      </c>
+      <c r="K30" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C31" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D31" t="n">
         <v>1240</v>
@@ -1388,19 +1583,25 @@
       <c r="H31" t="n">
         <v>0.114285714285714</v>
       </c>
-      <c r="I31" t="n">
-        <v>0.224551626023269</v>
+      <c r="I31" t="s">
+        <v>40</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.909337971369031</v>
+      </c>
+      <c r="K31" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B32" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D32" t="n">
         <v>1370</v>
@@ -1417,19 +1618,25 @@
       <c r="H32" t="n">
         <v>0.0714285714285714</v>
       </c>
-      <c r="I32" t="n">
-        <v>0.53752564534162</v>
+      <c r="I32" t="s">
+        <v>40</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.782975673296652</v>
+      </c>
+      <c r="K32" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D33" t="n">
         <v>1370</v>
@@ -1446,19 +1653,25 @@
       <c r="H33" t="n">
         <v>0.0714285714285714</v>
       </c>
-      <c r="I33" t="n">
-        <v>0.53752564534162</v>
+      <c r="I33" t="s">
+        <v>40</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.782975673296652</v>
+      </c>
+      <c r="K33" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B34" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D34" t="n">
         <v>1399</v>
@@ -1475,19 +1688,25 @@
       <c r="H34" t="n">
         <v>0.0571428571428571</v>
       </c>
-      <c r="I34" t="n">
-        <v>0.583081901833719</v>
+      <c r="I34" t="s">
+        <v>40</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.764582474799044</v>
+      </c>
+      <c r="K34" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D35" t="n">
         <v>1422</v>
@@ -1504,19 +1723,25 @@
       <c r="H35" t="n">
         <v>0.0428571428571429</v>
       </c>
-      <c r="I35" t="n">
-        <v>0.534322595906135</v>
+      <c r="I35" t="s">
+        <v>40</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.784268894658568</v>
+      </c>
+      <c r="K35" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D36" t="n">
         <v>1422</v>
@@ -1533,19 +1758,25 @@
       <c r="H36" t="n">
         <v>0.0428571428571429</v>
       </c>
-      <c r="I36" t="n">
-        <v>0.557787020752254</v>
+      <c r="I36" t="s">
+        <v>40</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.77479520526748</v>
+      </c>
+      <c r="K36" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B37" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
         <v>1444</v>
@@ -1562,8 +1793,14 @@
       <c r="H37" t="n">
         <v>0.0285714285714286</v>
       </c>
-      <c r="I37" t="n">
-        <v>0.392427363026869</v>
+      <c r="I37" t="s">
+        <v>40</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.841558658681764</v>
+      </c>
+      <c r="K37" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>